<commit_message>
Add changes to TestData.xlsx file.
</commit_message>
<xml_diff>
--- a/TDD/TestData.xlsx
+++ b/TDD/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\Claude\Printup project\TDD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15C3CC30-5C24-43C1-BEFF-7DF0871C7D5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5D13C84-1C13-4938-AAA5-11B76C2D96EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11625" yWindow="5535" windowWidth="23595" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11445" yWindow="2565" windowWidth="23595" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestData" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="137">
   <si>
     <t>ClientInfoFlow</t>
   </si>
@@ -238,9 +238,6 @@
     <t>15.4.2026</t>
   </si>
   <si>
-    <t>Approved</t>
-  </si>
-  <si>
     <t>רגיל</t>
   </si>
   <si>
@@ -262,9 +259,6 @@
     <t>22.3.2026</t>
   </si>
   <si>
-    <t>Not approved</t>
-  </si>
-  <si>
     <t>דחוף</t>
   </si>
   <si>
@@ -373,9 +367,6 @@
     <t>פרספקס לבן מבריק</t>
   </si>
   <si>
-    <t>כן</t>
-  </si>
-  <si>
     <t>PVC</t>
   </si>
   <si>
@@ -409,9 +400,6 @@
     <t>פולט אור שחור</t>
   </si>
   <si>
-    <t>לא</t>
-  </si>
-  <si>
     <t>פוליפלסט</t>
   </si>
   <si>
@@ -437,6 +425,12 @@
   </si>
   <si>
     <t>מדבקת ויניל מט</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>no</t>
   </si>
 </sst>
 </file>
@@ -1081,22 +1075,22 @@
         <v>71</v>
       </c>
       <c r="E17" t="s">
+        <v>135</v>
+      </c>
+      <c r="F17" t="s">
         <v>72</v>
-      </c>
-      <c r="F17" t="s">
-        <v>73</v>
       </c>
       <c r="G17">
         <v>0.33333333333333331</v>
       </c>
       <c r="H17" t="s">
+        <v>73</v>
+      </c>
+      <c r="I17" t="s">
         <v>74</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" t="s">
         <v>75</v>
-      </c>
-      <c r="J17" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -1104,31 +1098,31 @@
         <v>11</v>
       </c>
       <c r="B18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C18" t="s">
         <v>77</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>78</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
+        <v>136</v>
+      </c>
+      <c r="F18" t="s">
         <v>79</v>
-      </c>
-      <c r="E18" t="s">
-        <v>80</v>
-      </c>
-      <c r="F18" t="s">
-        <v>81</v>
       </c>
       <c r="G18">
         <v>0.4375</v>
       </c>
       <c r="H18" t="s">
+        <v>80</v>
+      </c>
+      <c r="I18" t="s">
+        <v>81</v>
+      </c>
+      <c r="J18" t="s">
         <v>82</v>
-      </c>
-      <c r="I18" t="s">
-        <v>83</v>
-      </c>
-      <c r="J18" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -1136,31 +1130,31 @@
         <v>16</v>
       </c>
       <c r="B19" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" t="s">
+        <v>84</v>
+      </c>
+      <c r="D19" t="s">
         <v>85</v>
       </c>
-      <c r="C19" t="s">
+      <c r="E19" t="s">
+        <v>135</v>
+      </c>
+      <c r="F19" t="s">
         <v>86</v>
-      </c>
-      <c r="D19" t="s">
-        <v>87</v>
-      </c>
-      <c r="E19" t="s">
-        <v>72</v>
-      </c>
-      <c r="F19" t="s">
-        <v>88</v>
       </c>
       <c r="G19">
         <v>0.54166666666666663</v>
       </c>
       <c r="H19" t="s">
+        <v>87</v>
+      </c>
+      <c r="I19" t="s">
+        <v>88</v>
+      </c>
+      <c r="J19" t="s">
         <v>89</v>
-      </c>
-      <c r="I19" t="s">
-        <v>90</v>
-      </c>
-      <c r="J19" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -1168,31 +1162,31 @@
         <v>21</v>
       </c>
       <c r="B20" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20" t="s">
+        <v>91</v>
+      </c>
+      <c r="D20" t="s">
         <v>92</v>
       </c>
-      <c r="C20" t="s">
-        <v>93</v>
-      </c>
-      <c r="D20" t="s">
-        <v>94</v>
-      </c>
       <c r="E20" t="s">
-        <v>80</v>
+        <v>136</v>
       </c>
       <c r="F20" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G20">
         <v>0.64583333333333337</v>
       </c>
       <c r="H20" t="s">
+        <v>93</v>
+      </c>
+      <c r="I20" t="s">
+        <v>94</v>
+      </c>
+      <c r="J20" t="s">
         <v>95</v>
-      </c>
-      <c r="I20" t="s">
-        <v>96</v>
-      </c>
-      <c r="J20" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -1200,192 +1194,192 @@
         <v>26</v>
       </c>
       <c r="B21" t="s">
+        <v>96</v>
+      </c>
+      <c r="C21" t="s">
+        <v>97</v>
+      </c>
+      <c r="D21" t="s">
         <v>98</v>
       </c>
-      <c r="C21" t="s">
-        <v>99</v>
-      </c>
-      <c r="D21" t="s">
-        <v>100</v>
-      </c>
       <c r="E21" t="s">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="F21" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G21">
         <v>0.375</v>
       </c>
       <c r="H21" t="s">
+        <v>99</v>
+      </c>
+      <c r="I21" t="s">
+        <v>100</v>
+      </c>
+      <c r="J21" t="s">
         <v>101</v>
-      </c>
-      <c r="I21" t="s">
-        <v>102</v>
-      </c>
-      <c r="J21" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" t="s">
         <v>105</v>
       </c>
-      <c r="B23" t="s">
+      <c r="D23" t="s">
         <v>106</v>
       </c>
-      <c r="C23" t="s">
+      <c r="E23" t="s">
+        <v>106</v>
+      </c>
+      <c r="F23" t="s">
         <v>107</v>
       </c>
-      <c r="D23" t="s">
+      <c r="G23" t="s">
         <v>108</v>
       </c>
-      <c r="E23" t="s">
-        <v>108</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="H23" t="s">
         <v>109</v>
-      </c>
-      <c r="G23" t="s">
-        <v>110</v>
-      </c>
-      <c r="H23" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B24">
         <v>8</v>
       </c>
       <c r="C24" t="s">
+        <v>111</v>
+      </c>
+      <c r="D24" t="s">
+        <v>112</v>
+      </c>
+      <c r="E24" t="s">
+        <v>72</v>
+      </c>
+      <c r="F24" t="s">
         <v>113</v>
       </c>
-      <c r="D24" t="s">
+      <c r="G24" t="s">
         <v>114</v>
       </c>
-      <c r="E24" t="s">
-        <v>73</v>
-      </c>
-      <c r="F24" t="s">
-        <v>115</v>
-      </c>
-      <c r="G24" t="s">
-        <v>116</v>
-      </c>
       <c r="H24" t="s">
-        <v>117</v>
+        <v>135</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B25">
         <v>4</v>
       </c>
       <c r="C25" t="s">
+        <v>116</v>
+      </c>
+      <c r="D25" t="s">
+        <v>111</v>
+      </c>
+      <c r="E25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F25" t="s">
+        <v>118</v>
+      </c>
+      <c r="G25" t="s">
         <v>119</v>
       </c>
-      <c r="D25" t="s">
-        <v>113</v>
-      </c>
-      <c r="E25" t="s">
-        <v>120</v>
-      </c>
-      <c r="F25" t="s">
-        <v>121</v>
-      </c>
-      <c r="G25" t="s">
-        <v>122</v>
-      </c>
       <c r="H25" t="s">
-        <v>117</v>
+        <v>135</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B26">
         <v>6</v>
       </c>
       <c r="C26" t="s">
+        <v>121</v>
+      </c>
+      <c r="D26" t="s">
+        <v>122</v>
+      </c>
+      <c r="E26" t="s">
+        <v>123</v>
+      </c>
+      <c r="F26" t="s">
         <v>124</v>
       </c>
-      <c r="D26" t="s">
+      <c r="G26" t="s">
         <v>125</v>
       </c>
-      <c r="E26" t="s">
-        <v>126</v>
-      </c>
-      <c r="F26" t="s">
-        <v>127</v>
-      </c>
-      <c r="G26" t="s">
-        <v>128</v>
-      </c>
       <c r="H26" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B27">
         <v>6</v>
       </c>
       <c r="C27" t="s">
+        <v>127</v>
+      </c>
+      <c r="D27" t="s">
+        <v>128</v>
+      </c>
+      <c r="E27" t="s">
+        <v>129</v>
+      </c>
+      <c r="F27" t="s">
+        <v>130</v>
+      </c>
+      <c r="G27" t="s">
         <v>131</v>
       </c>
-      <c r="D27" t="s">
-        <v>132</v>
-      </c>
-      <c r="E27" t="s">
-        <v>133</v>
-      </c>
-      <c r="F27" t="s">
-        <v>134</v>
-      </c>
-      <c r="G27" t="s">
+      <c r="H27" t="s">
         <v>135</v>
-      </c>
-      <c r="H27" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B28">
         <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D28" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E28" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F28" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G28" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="H28" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -1403,7 +1397,7 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I1 A22:I23 A3:I15 B2:I2 A28:E28 A24:E24 G24:I24 A25:E25 G25:I25 A26:E26 G26:I26 A27:E27 G27:I27 G28:I28" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:I1 A22:I23 A3:I15 B2:I2 A28:E28 A24:E24 G24 A25:E25 G25 A26:E26 G26 A27:E27 G27 G28 I24 I25 I26 I27 I28" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>